<commit_message>
feat: implement auto-execution of precondition operation codes in PreconditionService
</commit_message>
<xml_diff>
--- a/docs/销售出库测试用例.xlsx
+++ b/docs/销售出库测试用例.xlsx
@@ -1,46 +1,208 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huhu/project/weberpagent/docs/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868D45A8-AE13-B945-BC4A-653746E78575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="测试用例" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
+  <si>
+    <t>任务名称</t>
+  </si>
+  <si>
+    <t>登录角色</t>
+  </si>
+  <si>
+    <t>任务描述</t>
+  </si>
+  <si>
+    <t>目标URL</t>
+  </si>
+  <si>
+    <t>最大步数</t>
+  </si>
+  <si>
+    <t>前置条件</t>
+  </si>
+  <si>
+    <t>断言</t>
+  </si>
+  <si>
+    <t>销售出库-未收款测试</t>
+  </si>
+  <si>
+    <t>main</t>
+  </si>
+  <si>
+    <t>步骤1：{点击}库存管理
+步骤2：{点击}出库管理
+步骤3：{点击}销售出库
+步骤4：{点击}请选择客户{选择第二个，并确认已显示所选客户名称}
+步骤5：{点击}物品编号{调用方法获取数据：{{imei}}，并确认输入框中已存在该编号}
+步骤6：{点击}添加{点击后必须确认列表中已出现该 imei 对应商品行；若列表仍显示"暂无数据"或未出现该商品行，则等待后重试，不要直接进入下一步}
+步骤7：{输入}列表中的：{销售金额}{150}
+要求：必须在包含 {{imei}} 的商品行中填写"销售金额"=150，不要填写其他金额输入框。
+填写后必须确认该商品行的销售金额已显示为 150 或 150.00；若未生效，继续定位该商品行中的销售金额输入框重试，不要跳过此步骤。
+步骤8：{输入}请输入物流单号{输入随机物流单号，并确认已输入成功}
+步骤9：{输入}请输入物流费用{10，并确认字段值为10或10.00}
+步骤10：{点击}收款信息{若收款信息区域已展开则无需重复点击}
+步骤11：{点击}是否收款 - 未收款{点击后确认"未收款"已被选中，且不是"已收款"}
+步骤12：{点击}确认
+要求：点击前再次确认以下关键字段：
+1. 列表中商品为 {{imei}}
+2. 销售金额 = 150
+3. 物流费用 = 10
+4. 金额 = 10
+5. 收款状态 = 未收款
+确认无误后再点击"确认"。</t>
+  </si>
+  <si>
+    <t>https://erptest.epbox.cn/</t>
+  </si>
+  <si>
+    <t>["context['preconditions'] = ['ekBx', 'wQ7u']", "items = context.get_data('PcImport', '库存管理|库存列表', i=2, j=13)\ncontext['imei'] = items[0]['imei']"]</t>
+  </si>
+  <si>
+    <t>[{"className": "PcAssert", "methodName": "bfCKxO", "headers": "main", "field_params": {"salesOrder": "SA", "articlesStateStr": "已销售", "saleTime": "now"}}]</t>
+  </si>
+  <si>
+    <t>销售出库-未收款-上传文件测试</t>
+  </si>
+  <si>
+    <t>步骤1：{点击}库存管理
+步骤2：{点击}出库管理
+步骤3：{点击}销售出库
+步骤4：{点击}请选择客户{选择第二个，并确认已显示所选客户名称}
+步骤5：{点击}导入添加
+步骤6：{上传}excel文件{{excel_file}}
+步骤7: {点击}确定 {确保成功新增一条数据}
+步骤8：{输入}列表中的：{销售金额}{150}
+要求：必须在商品行中填写"销售金额"=150，不要填写其他金额输入框。
+填写后必须确认该商品行的销售金额已显示为 150 或 150.00；若未生效，继续定位该商品行中的销售金额输入框重试，不要跳过此步骤。
+步骤9：{输入}请输入物流单号{输入随机物流单号，并确认已输入成功}
+步骤10：{输入}请输入物流费用{10，并确认字段值为10或10.00}
+步骤11：{点击}收款信息{若收款信息区域已展开则无需重复点击}
+步骤12：{点击}是否收款 - 未收款{点击后确认"未收款"已被选中，且不是"已收款"}
+步骤13：{点击}确认
+要求：点击前再次确认以下关键字段：
+1. 列表中商品存在
+2. 销售金额 = 150
+3. 物流费用 = 10
+4. 金额 = 10
+5. 收款状态 = 未收款
+确认无误后再点击"确认"。</t>
+  </si>
+  <si>
+    <t>["context['preconditions'] = ['ekBx', 'wQ7u']", "items = context.get_data('PcImport', '库存管理|库存列表', i=2, j=13)\ncontext.fill_excel('new_purchase_order', row=2, col=1, value=items[0]['imei'])\ncontext['excel_file'] = context.get_excel_path('new_purchase_order')"]</t>
+  </si>
+  <si>
+    <t>库存列表-物品详情点击测试</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>main</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://erptest.epbox.cn/</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. {点击} 库存管理
+2. {点击} 库存列表
+3. {点击} 物品编号的第一行物品
+4. {确认} 进入物品详情页面</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>隐藏元素测试</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. {点击} 商品采购
+2. {点击} 采购管理
+3. {点击} 采购工单
+4. {点击} 工单列表第一行工单 {操作列} 的{更多}
+5. {点击} 报工明细
+6. {确认} 弹出报功明细</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>双击修改测试</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. {点击} 库存管理
+2. {点击} 库存列表
+3. {双击} 物品列表的 {IMEI号}的第一行
+4. {输入} shuangjiceshi
+5. {点击} 任意空白区域
+6.{确认} 修改成功</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4">
     <font>
-      <name val="Calibri"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="宋体"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003B82F6"/>
-        <bgColor rgb="003B82F6"/>
+        <fgColor rgb="FF3B82F6"/>
+        <bgColor rgb="FF3B82F6"/>
       </patternFill>
     </fill>
   </fills>
@@ -53,96 +215,52 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="超链接" xfId="1" builtinId="8"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -430,116 +548,146 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="80" customWidth="1"/>
+    <col min="4" max="4" width="35" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="7" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>任务名称</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>登录角色</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>任务描述</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>目标URL</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>最大步数</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>前置条件</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>断言</t>
-        </is>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="2" ht="400" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>销售出库-未收款测试</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>步骤1：{点击}库存管理
-步骤2：{点击}出库管理
-步骤3：{点击}销售出库
-步骤4：{点击}请选择客户{选择第二个，并确认已显示所选客户名称}
-步骤5：{点击}物品编号{调用方法获取数据：{{imei}}，并确认输入框中已存在该编号}
-步骤6：{点击}添加{点击后必须确认列表中已出现该 imei 对应商品行；若列表仍显示"暂无数据"或未出现该商品行，则等待后重试，不要直接进入下一步}
-步骤7：{输入}列表中的：{销售金额}{150}
-要求：必须在包含 {{imei}} 的商品行中填写"销售金额"=150，不要填写其他金额输入框。
-填写后必须确认该商品行的销售金额已显示为 150 或 150.00；若未生效，继续定位该商品行中的销售金额输入框重试，不要跳过此步骤。
-步骤8：{输入}请输入物流单号{输入随机物流单号，并确认已输入成功}
-步骤9：{输入}请输入物流费用{10，并确认字段值为10或10.00}
-步骤10：{点击}收款信息{若收款信息区域已展开则无需重复点击}
-步骤11：{点击}是否收款 - 未收款{点击后确认"未收款"已被选中，且不是"已收款"}
-步骤12：{点击}确认
-要求：点击前再次确认以下关键字段：
-1. 列表中商品为 {{imei}}
-2. 销售金额 = 150
-3. 物流费用 = 10
-4. 金额 = 10
-5. 收款状态 = 未收款
-确认无误后再点击"确认"。</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>https://erptest.epbox.cn/</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n">
+    <row r="2" spans="1:7" ht="400" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="2">
         <v>20</v>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>["context['preconditions'] = ['FA1', 'HC1']", "items = context.get_data('PcImport', '库存管理|库存列表', i=2, j=13)\ncontext['imei'] = items[0]['imei']"]</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>[{"methodName": "sell_sale_item_list_assert", "headers": "main", "params": {"salesOrder": "SA", "articlesStateStr": "已销售", "saleTime": "now"}}]</t>
-        </is>
+      <c r="F2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="342" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="2">
+        <v>20</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="60">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="90">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="90">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D4" r:id="rId2" xr:uid="{2F9E6856-EF1B-0C43-A633-738F39386F98}"/>
+    <hyperlink ref="D5" r:id="rId3" xr:uid="{A2C1E269-4A24-B045-9AE9-39615CB109A5}"/>
+    <hyperlink ref="D6" r:id="rId4" xr:uid="{80561E39-DAF2-B543-BF6E-1BC26E92E004}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>